<commit_message>
feat: add coverage ledger tool and update JD library template
</commit_message>
<xml_diff>
--- a/templates/jd-library.template.xlsx
+++ b/templates/jd-library.template.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI1"/>
+  <dimension ref="A1:AJ1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -456,7 +456,7 @@
     <col width="16" customWidth="1" min="32" max="32"/>
     <col width="16" customWidth="1" min="33" max="33"/>
     <col width="16" customWidth="1" min="34" max="34"/>
-    <col width="16" customWidth="1" min="35" max="35"/>
+    <col width="22" customWidth="1" min="35" max="35"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -631,6 +631,11 @@
         </is>
       </c>
       <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>全部来源</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>备注/质量说明</t>
         </is>
@@ -647,7 +652,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AK1"/>
+  <dimension ref="A1:AL1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -684,7 +689,7 @@
     <col width="16" customWidth="1" min="32" max="32"/>
     <col width="16" customWidth="1" min="33" max="33"/>
     <col width="16" customWidth="1" min="34" max="34"/>
-    <col width="16" customWidth="1" min="35" max="35"/>
+    <col width="22" customWidth="1" min="35" max="35"/>
     <col width="16" customWidth="1" min="36" max="36"/>
     <col width="16" customWidth="1" min="37" max="37"/>
   </cols>
@@ -862,15 +867,20 @@
       </c>
       <c r="AI1" s="1" t="inlineStr">
         <is>
+          <t>全部来源</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
           <t>备注/质量说明</t>
         </is>
       </c>
-      <c r="AJ1" s="1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>失效日期</t>
         </is>
       </c>
-      <c r="AK1" s="1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>失效原因</t>
         </is>
@@ -887,13 +897,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:D1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
@@ -910,15 +920,10 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>旧值</t>
+          <t>统计</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>新值</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>原因</t>
         </is>

</xml_diff>